<commit_message>
Updated Potentail Verification Tests
</commit_message>
<xml_diff>
--- a/docs/project_plan.xlsx
+++ b/docs/project_plan.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10320"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keanu\Desktop\CS2430\project2\2430_501_Team6_Project2\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keanu\Desktop\CS2430\project3\Programming_Project_3\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32DC036C-06B7-411D-8CE8-07D4D1F89A1B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEED74C9-23CD-4E9E-8A99-620F78CF7A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Info" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="112" uniqueCount="117">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="112">
   <si>
     <t>CSIS 2430 — Project Plan (Plan + Trace)</t>
   </si>
@@ -282,9 +282,6 @@
     <t>Repository URL: https://github.com/jmack02-ui/Programming_Project_3</t>
   </si>
   <si>
-    <t>Instructor invited as viewer by checkpoint?: NO //TODO</t>
-  </si>
-  <si>
     <t>Project2/src/* Owned by Implementation Lead.</t>
   </si>
   <si>
@@ -303,13 +300,85 @@
     <t>Part II - Tests for Brute Force Strategies</t>
   </si>
   <si>
-    <t>Part III - Dynamic Programming (Optional)</t>
-  </si>
-  <si>
-    <t>TBD</t>
-  </si>
-  <si>
     <t>Commits are never made to made to the main branch. Work is committed in separate branches, then merged through PR into main.</t>
+  </si>
+  <si>
+    <t>Instructor invited as viewer by checkpoint?: YES Invited 3/28/2026</t>
+  </si>
+  <si>
+    <t>Highest Rating Does Not Exceed Bounds</t>
+  </si>
+  <si>
+    <t>Lightest Weight Does Not Exceed Bounds</t>
+  </si>
+  <si>
+    <t>Empty Experiment List</t>
+  </si>
+  <si>
+    <t>All Experiments Too Heavy</t>
+  </si>
+  <si>
+    <t>Standard Expected Operation</t>
+  </si>
+  <si>
+    <t>High Rating High Weight</t>
+  </si>
+  <si>
+    <t>Low Weight Low Rating</t>
+  </si>
+  <si>
+    <t>Part IV - Dynamic Programming (Optional)</t>
+  </si>
+  <si>
+    <t>Part III - Comparison Output</t>
+  </si>
+  <si>
+    <t>Output Works As Intended</t>
+  </si>
+  <si>
+    <t>Optimal Case Check</t>
+  </si>
+  <si>
+    <t>Subset Count Validation</t>
+  </si>
+  <si>
+    <t>Less than 3 Subsets</t>
+  </si>
+  <si>
+    <t>Multiple Subsets Same Rating</t>
+  </si>
+  <si>
+    <t>Subsets Within Weight Bounds</t>
+  </si>
+  <si>
+    <t>Same Weight Same Rating Multiple Items</t>
+  </si>
+  <si>
+    <t>Same Ratio Multiple Items</t>
+  </si>
+  <si>
+    <t>Sort Order Consistency</t>
+  </si>
+  <si>
+    <t>Correct Totals</t>
+  </si>
+  <si>
+    <t>Correct Experiment Outputs</t>
+  </si>
+  <si>
+    <t>Does Not Divide by Zero</t>
+  </si>
+  <si>
+    <t>No Valid Subsets</t>
+  </si>
+  <si>
+    <t>Greedy Fails Vs Brute Force</t>
+  </si>
+  <si>
+    <t>Matches Brute Force Optimal</t>
+  </si>
+  <si>
+    <t>Handles Large Dataset</t>
   </si>
 </sst>
 </file>
@@ -319,7 +388,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="16" x14ac:knownFonts="1">
+  <fonts count="14" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -416,27 +485,13 @@
     </font>
     <font>
       <sz val="11"/>
-      <color rgb="FFFF0000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="11"/>
-      <color theme="3" tint="0.39997558519241921"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <charset val="1"/>
-    </font>
-    <font>
-      <sz val="15"/>
-      <color theme="3" tint="0.39997558519241921"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="5">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -453,12 +508,6 @@
       <patternFill patternType="solid">
         <fgColor rgb="FF1F4E79"/>
         <bgColor rgb="FF1F497D"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="0"/>
-        <bgColor indexed="64"/>
       </patternFill>
     </fill>
     <fill>
@@ -588,7 +637,7 @@
     <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="58">
+  <cellXfs count="54">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -706,49 +755,37 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="4" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="5" borderId="0" xfId="3" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
   </cellXfs>
@@ -1020,27 +1057,27 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F32"/>
-  <sheetFormatPr defaultColWidth="8.609375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="40.22265625" style="1" customWidth="1"/>
-    <col min="2" max="2" width="34.03125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="39.68359375" style="1" customWidth="1"/>
-    <col min="4" max="4" width="27.98046875" style="1" customWidth="1"/>
-    <col min="5" max="6" width="18.0234375" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.609375" style="1"/>
+    <col min="1" max="1" width="40.19921875" style="1" customWidth="1"/>
+    <col min="2" max="2" width="34" style="1" customWidth="1"/>
+    <col min="3" max="3" width="39.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="28" style="1" customWidth="1"/>
+    <col min="5" max="6" width="18" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.59765625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="18.75" x14ac:dyDescent="0.2">
-      <c r="A1" s="42" t="s">
+    <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.45">
+      <c r="A1" s="47" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="42"/>
-      <c r="C1" s="42"/>
-      <c r="D1" s="42"/>
-      <c r="E1" s="42"/>
-      <c r="F1" s="42"/>
-    </row>
-    <row r="3" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+    </row>
+    <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
         <v>1</v>
       </c>
@@ -1050,12 +1087,12 @@
       <c r="E3" s="3"/>
       <c r="F3" s="3"/>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
         <v>70</v>
       </c>
@@ -1065,7 +1102,7 @@
       <c r="E5" s="43"/>
       <c r="F5" s="43"/>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>71</v>
       </c>
@@ -1075,7 +1112,7 @@
       <c r="E6" s="43"/>
       <c r="F6" s="43"/>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
         <v>72</v>
       </c>
@@ -1085,7 +1122,7 @@
       <c r="E7" s="43"/>
       <c r="F7" s="43"/>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
         <v>73</v>
       </c>
@@ -1095,7 +1132,7 @@
       <c r="E8" s="43"/>
       <c r="F8" s="43"/>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
         <v>74</v>
       </c>
@@ -1105,7 +1142,7 @@
       <c r="E9" s="43"/>
       <c r="F9" s="43"/>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="4"/>
       <c r="B10" s="43"/>
       <c r="C10" s="43"/>
@@ -1113,17 +1150,17 @@
       <c r="E10" s="43"/>
       <c r="F10" s="43"/>
     </row>
-    <row r="11" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
-      <c r="A11" s="44" t="s">
+    <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.45">
+      <c r="A11" s="46" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="44"/>
-      <c r="C11" s="44"/>
-      <c r="D11" s="44"/>
-      <c r="E11" s="44"/>
-      <c r="F11" s="44"/>
-    </row>
-    <row r="12" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B11" s="46"/>
+      <c r="C11" s="46"/>
+      <c r="D11" s="46"/>
+      <c r="E11" s="46"/>
+      <c r="F11" s="46"/>
+    </row>
+    <row r="12" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="43" t="s">
         <v>4</v>
       </c>
@@ -1133,8 +1170,8 @@
       <c r="E12" s="43"/>
       <c r="F12" s="43"/>
     </row>
-    <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.2"/>
-    <row r="14" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="14" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="5" t="s">
         <v>5</v>
       </c>
@@ -1148,7 +1185,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="15" spans="1:6" s="41" customFormat="1" ht="44.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
         <v>77</v>
       </c>
@@ -1160,7 +1197,7 @@
       </c>
       <c r="D15" s="5"/>
     </row>
-    <row r="16" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
         <v>76</v>
       </c>
@@ -1172,7 +1209,7 @@
       </c>
       <c r="D16" s="5"/>
     </row>
-    <row r="17" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" ht="51" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="5" t="s">
         <v>11</v>
       </c>
@@ -1186,7 +1223,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="18" spans="1:4" ht="56.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" ht="56.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="5" t="s">
         <v>75</v>
       </c>
@@ -1198,88 +1235,103 @@
       </c>
       <c r="D18" s="5"/>
     </row>
-    <row r="19" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="45" t="s">
+    <row r="19" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="44" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="45"/>
-    </row>
-    <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B19" s="44"/>
+    </row>
+    <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="43" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="43"/>
     </row>
-    <row r="21" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A21" s="43" t="s">
         <v>78</v>
       </c>
       <c r="B21" s="43"/>
     </row>
-    <row r="22" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A22" s="50" t="s">
-        <v>79</v>
+        <v>86</v>
       </c>
       <c r="B22" s="50"/>
     </row>
-    <row r="23" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" s="43" t="s">
         <v>19</v>
       </c>
       <c r="B23" s="43"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="43"/>
       <c r="B24" s="43"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A25" s="45" t="s">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A25" s="44" t="s">
         <v>20</v>
       </c>
-      <c r="B25" s="45"/>
-    </row>
-    <row r="26" spans="1:4" ht="41.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A26" s="47" t="s">
-        <v>88</v>
-      </c>
-      <c r="B26" s="47"/>
-    </row>
-    <row r="27" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A27" s="45" t="s">
+      <c r="B25" s="44"/>
+    </row>
+    <row r="26" spans="1:4" ht="41.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A26" s="45" t="s">
+        <v>85</v>
+      </c>
+      <c r="B26" s="45"/>
+    </row>
+    <row r="27" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A27" s="44" t="s">
         <v>21</v>
       </c>
-      <c r="B27" s="45"/>
-    </row>
-    <row r="28" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A28" s="47" t="s">
+      <c r="B27" s="44"/>
+    </row>
+    <row r="28" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A28" s="45" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="47"/>
-    </row>
-    <row r="29" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A29" s="46" t="s">
+      <c r="B28" s="45"/>
+    </row>
+    <row r="29" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="42" t="s">
+        <v>79</v>
+      </c>
+      <c r="B29" s="42"/>
+    </row>
+    <row r="30" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="42" t="s">
         <v>80</v>
       </c>
-      <c r="B29" s="46"/>
-    </row>
-    <row r="30" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A30" s="46" t="s">
-        <v>81</v>
-      </c>
-      <c r="B30" s="46"/>
-    </row>
-    <row r="31" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.15">
-      <c r="A31" s="46" t="s">
+      <c r="B30" s="42"/>
+    </row>
+    <row r="31" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="42" t="s">
         <v>23</v>
       </c>
-      <c r="B31" s="46"/>
-    </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="B31" s="42"/>
+    </row>
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="43"/>
       <c r="B32" s="43"/>
     </row>
   </sheetData>
   <mergeCells count="23">
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A32:B32"/>
@@ -1288,21 +1340,6 @@
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A29:B29"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B8:F8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1312,17 +1349,17 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:F9"/>
-  <sheetFormatPr defaultColWidth="8.609375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="34.03125" customWidth="1"/>
-    <col min="2" max="2" width="13.98828125" style="6" customWidth="1"/>
-    <col min="3" max="3" width="13.98828125" customWidth="1"/>
-    <col min="4" max="4" width="43.98828125" style="7" customWidth="1"/>
-    <col min="5" max="5" width="13.98828125" customWidth="1"/>
-    <col min="6" max="6" width="29.99609375" customWidth="1"/>
+    <col min="1" max="1" width="34" customWidth="1"/>
+    <col min="2" max="2" width="14" style="6" customWidth="1"/>
+    <col min="3" max="3" width="14" customWidth="1"/>
+    <col min="4" max="4" width="44" style="7" customWidth="1"/>
+    <col min="5" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A1" s="48" t="s">
         <v>24</v>
       </c>
@@ -1332,7 +1369,7 @@
       <c r="E1" s="48"/>
       <c r="F1" s="48"/>
     </row>
-    <row r="2" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="49" t="s">
         <v>25</v>
       </c>
@@ -1342,7 +1379,7 @@
       <c r="E2" s="49"/>
       <c r="F2" s="49"/>
     </row>
-    <row r="4" spans="1:6" ht="27" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" ht="27" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
         <v>26</v>
       </c>
@@ -1362,7 +1399,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="10" t="s">
         <v>32</v>
       </c>
@@ -1370,7 +1407,7 @@
         <v>46110</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D5" s="10" t="s">
         <v>33</v>
@@ -1378,7 +1415,7 @@
       <c r="E5" s="12"/>
       <c r="F5" s="10"/>
     </row>
-    <row r="6" spans="1:6" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A6" s="10" t="s">
         <v>34</v>
       </c>
@@ -1386,7 +1423,7 @@
         <v>46117</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D6" s="10" t="s">
         <v>35</v>
@@ -1394,7 +1431,7 @@
       <c r="E6" s="12"/>
       <c r="F6" s="10"/>
     </row>
-    <row r="7" spans="1:6" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A7" s="10" t="s">
         <v>36</v>
       </c>
@@ -1410,7 +1447,7 @@
       <c r="E7" s="12"/>
       <c r="F7" s="10"/>
     </row>
-    <row r="8" spans="1:6" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A8" s="10" t="s">
         <v>38</v>
       </c>
@@ -1418,7 +1455,7 @@
         <v>46123</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D8" s="10" t="s">
         <v>40</v>
@@ -1426,7 +1463,7 @@
       <c r="E8" s="12"/>
       <c r="F8" s="10"/>
     </row>
-    <row r="9" spans="1:6" ht="27.75" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A9" s="10" t="s">
         <v>41</v>
       </c>
@@ -1434,7 +1471,7 @@
         <v>46124</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D9" s="10" t="s">
         <v>42</v>
@@ -1461,16 +1498,16 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:G18"/>
-  <sheetFormatPr defaultColWidth="8.609375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="6.05078125" customWidth="1"/>
-    <col min="2" max="2" width="45.87109375" style="7" customWidth="1"/>
-    <col min="3" max="5" width="13.98828125" customWidth="1"/>
-    <col min="6" max="6" width="29.45703125" style="36" customWidth="1"/>
-    <col min="7" max="7" width="29.99609375" customWidth="1"/>
+    <col min="1" max="1" width="6.06640625" customWidth="1"/>
+    <col min="2" max="2" width="45.86328125" style="7" customWidth="1"/>
+    <col min="3" max="5" width="14" customWidth="1"/>
+    <col min="6" max="6" width="29.46484375" style="36" customWidth="1"/>
+    <col min="7" max="7" width="30" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A1" s="48" t="s">
         <v>43</v>
       </c>
@@ -1481,7 +1518,7 @@
       <c r="F1" s="48"/>
       <c r="G1" s="48"/>
     </row>
-    <row r="2" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="49" t="s">
         <v>44</v>
       </c>
@@ -1492,7 +1529,7 @@
       <c r="F2" s="49"/>
       <c r="G2" s="49"/>
     </row>
-    <row r="4" spans="1:7" ht="27" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:7" ht="27" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
         <v>45</v>
       </c>
@@ -1515,7 +1552,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="14">
         <v>1</v>
       </c>
@@ -1523,7 +1560,7 @@
         <v>49</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D5" s="16">
         <v>46110</v>
@@ -1532,7 +1569,7 @@
       <c r="F5" s="31"/>
       <c r="G5" s="15"/>
     </row>
-    <row r="6" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="14">
         <v>2</v>
       </c>
@@ -1540,7 +1577,7 @@
         <v>50</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D6" s="16">
         <v>46117</v>
@@ -1549,7 +1586,7 @@
       <c r="F6" s="32"/>
       <c r="G6" s="15"/>
     </row>
-    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="14">
         <v>3</v>
       </c>
@@ -1557,7 +1594,7 @@
         <v>51</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D7" s="16">
         <v>46123</v>
@@ -1566,7 +1603,7 @@
       <c r="F7" s="32"/>
       <c r="G7" s="15"/>
     </row>
-    <row r="8" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="14">
         <v>4</v>
       </c>
@@ -1574,7 +1611,7 @@
         <v>52</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D8" s="16">
         <v>46123</v>
@@ -1583,7 +1620,7 @@
       <c r="F8" s="33"/>
       <c r="G8" s="15"/>
     </row>
-    <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="14">
         <v>5</v>
       </c>
@@ -1600,7 +1637,7 @@
       <c r="F9" s="34"/>
       <c r="G9" s="15"/>
     </row>
-    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="14">
         <v>6</v>
       </c>
@@ -1617,7 +1654,7 @@
       <c r="F10" s="34"/>
       <c r="G10" s="15"/>
     </row>
-    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="14">
         <v>7</v>
       </c>
@@ -1634,7 +1671,7 @@
       <c r="F11" s="34"/>
       <c r="G11" s="15"/>
     </row>
-    <row r="12" spans="1:7" ht="26.85" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:7" ht="26.85" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="14">
         <v>8</v>
       </c>
@@ -1651,7 +1688,7 @@
       <c r="F12" s="34"/>
       <c r="G12" s="15"/>
     </row>
-    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="14">
         <v>9</v>
       </c>
@@ -1659,7 +1696,7 @@
         <v>56</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D13" s="16">
         <v>46110</v>
@@ -1668,7 +1705,7 @@
       <c r="F13" s="34"/>
       <c r="G13" s="15"/>
     </row>
-    <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="14">
         <v>10</v>
       </c>
@@ -1676,7 +1713,7 @@
         <v>57</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D14" s="16">
         <v>46117</v>
@@ -1685,7 +1722,7 @@
       <c r="F14" s="34"/>
       <c r="G14" s="15"/>
     </row>
-    <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="14">
         <v>11</v>
       </c>
@@ -1693,7 +1730,7 @@
         <v>58</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D15" s="16">
         <v>46117</v>
@@ -1702,7 +1739,7 @@
       <c r="F15" s="34"/>
       <c r="G15" s="15"/>
     </row>
-    <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="19">
         <v>12</v>
       </c>
@@ -1710,7 +1747,7 @@
         <v>59</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D16" s="16">
         <v>46124</v>
@@ -1719,7 +1756,7 @@
       <c r="F16" s="34"/>
       <c r="G16" s="15"/>
     </row>
-    <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="15"/>
       <c r="B17" s="20"/>
       <c r="C17" s="21"/>
@@ -1728,7 +1765,7 @@
       <c r="F17" s="35"/>
       <c r="G17" s="22"/>
     </row>
-    <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="15"/>
       <c r="B18" s="18"/>
       <c r="C18" s="15"/>
@@ -1749,134 +1786,187 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:B36"/>
-  <sheetFormatPr defaultColWidth="8.609375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="A1:B39"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="72.23828125" style="7" customWidth="1"/>
-    <col min="2" max="2" width="18.96484375" customWidth="1"/>
-    <col min="3" max="4" width="9.953125" customWidth="1"/>
+    <col min="1" max="1" width="72.265625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="18.9296875" customWidth="1"/>
+    <col min="3" max="4" width="9.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" ht="19.5" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:2" ht="19.5" x14ac:dyDescent="0.6">
       <c r="A1" s="24" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="41" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" s="41" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" s="41" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" s="41" t="s">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" s="41" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" s="41" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" s="41" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A9" s="41" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A10" s="41" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A11" s="41" t="s">
+        <v>103</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A12" s="53" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A13" s="24" t="s">
         <v>84</v>
       </c>
     </row>
-    <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="54" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A3" s="54"/>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A4" s="54"/>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A5" s="54"/>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A6" s="54"/>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A7" s="54"/>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A8" s="54"/>
-    </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A9" s="55"/>
-    </row>
-    <row r="10" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="24" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="56" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A12" s="57"/>
-      <c r="B12" s="25"/>
-    </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A13" s="56"/>
-    </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A14" s="56"/>
-    </row>
-    <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A15" s="56"/>
-    </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
-      <c r="A16" s="56"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A17" s="56"/>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A18" s="57"/>
-    </row>
-    <row r="19" spans="1:1" ht="23.25" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A19" s="24" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="20" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A20" s="56" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="21" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A21" s="56"/>
-    </row>
-    <row r="22" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A22" s="56"/>
-    </row>
-    <row r="23" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A23" s="56"/>
-    </row>
-    <row r="24" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A24" s="56"/>
-    </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A25" s="56"/>
-    </row>
-    <row r="26" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A26" s="56"/>
-    </row>
-    <row r="27" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A27" s="57"/>
-    </row>
-    <row r="28" spans="1:1" ht="21.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="53"/>
-    </row>
-    <row r="29" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="51" t="s">
+        <v>91</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="52" t="s">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A16" s="51" t="s">
+        <v>97</v>
+      </c>
+      <c r="B16" s="25"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A17" s="51" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A18" s="51" t="s">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="51" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="20" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A20" s="51" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A21" s="52"/>
+    </row>
+    <row r="22" spans="1:1" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A22" s="24" t="s">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="51" t="s">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A24" s="51" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A25" s="51" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A26" s="51" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A27" s="51"/>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A28" s="51"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A29" s="51"/>
     </row>
-    <row r="30" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A30" s="51"/>
-    </row>
-    <row r="31" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A31" s="51"/>
-    </row>
-    <row r="32" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A32" s="51"/>
-    </row>
-    <row r="33" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A33" s="51"/>
-    </row>
-    <row r="34" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A30" s="52"/>
+    </row>
+    <row r="31" spans="1:1" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
+      <c r="A31" s="24" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" ht="21.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A32" s="51" t="s">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="33" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A33" s="51" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A34" s="51"/>
     </row>
-    <row r="35" spans="1:1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:1" x14ac:dyDescent="0.45">
       <c r="A35" s="51"/>
     </row>
-    <row r="36" spans="1:1" x14ac:dyDescent="0.2">
-      <c r="A36" s="52"/>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A36" s="51"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A37" s="51"/>
+    </row>
+    <row r="38" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A38" s="51"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A39" s="52"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1887,16 +1977,16 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:E6"/>
-  <sheetFormatPr defaultColWidth="8.609375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="29.99609375" customWidth="1"/>
-    <col min="2" max="2" width="11.97265625" customWidth="1"/>
-    <col min="3" max="3" width="43.98828125" customWidth="1"/>
-    <col min="4" max="4" width="13.98828125" customWidth="1"/>
-    <col min="5" max="5" width="11.97265625" customWidth="1"/>
+    <col min="1" max="1" width="30" customWidth="1"/>
+    <col min="2" max="2" width="12" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
+    <col min="4" max="4" width="14" customWidth="1"/>
+    <col min="5" max="5" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:5" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A1" s="48" t="s">
         <v>60</v>
       </c>
@@ -1905,7 +1995,7 @@
       <c r="D1" s="48"/>
       <c r="E1" s="48"/>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
         <v>61</v>
       </c>
@@ -1922,21 +2012,21 @@
         <v>64</v>
       </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="26"/>
       <c r="B4" s="26"/>
       <c r="C4" s="26"/>
       <c r="D4" s="26"/>
       <c r="E4" s="26"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="26"/>
       <c r="B5" s="26"/>
       <c r="C5" s="26"/>
       <c r="D5" s="26"/>
       <c r="E5" s="26"/>
     </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="26"/>
       <c r="B6" s="26"/>
       <c r="C6" s="26"/>
@@ -1955,15 +2045,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:D33"/>
-  <sheetFormatPr defaultColWidth="8.609375" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.59765625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="13.98828125" customWidth="1"/>
-    <col min="2" max="2" width="52.05859375" customWidth="1"/>
-    <col min="3" max="3" width="34.03125" customWidth="1"/>
-    <col min="4" max="4" width="28.921875" style="36" customWidth="1"/>
+    <col min="1" max="1" width="14" customWidth="1"/>
+    <col min="2" max="2" width="52.06640625" customWidth="1"/>
+    <col min="3" max="3" width="34" customWidth="1"/>
+    <col min="4" max="4" width="28.9296875" style="36" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="15.75" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
       <c r="A1" s="48" t="s">
         <v>65</v>
       </c>
@@ -1971,7 +2061,7 @@
       <c r="C1" s="48"/>
       <c r="D1" s="48"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="27" t="s">
         <v>66</v>
       </c>
@@ -1985,181 +2075,181 @@
         <v>69</v>
       </c>
     </row>
-    <row r="4" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="28"/>
       <c r="B4" s="29"/>
       <c r="C4" s="29"/>
       <c r="D4" s="38"/>
     </row>
-    <row r="5" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="28"/>
       <c r="B5" s="29"/>
       <c r="C5" s="29"/>
       <c r="D5" s="38"/>
     </row>
-    <row r="6" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="28"/>
       <c r="B6" s="29"/>
       <c r="C6" s="29"/>
       <c r="D6" s="39"/>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="28"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
       <c r="D7" s="39"/>
     </row>
-    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
       <c r="D8" s="39"/>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
       <c r="D9" s="39"/>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
       <c r="D10" s="40"/>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="40"/>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="40"/>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="40"/>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="40"/>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="40"/>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="40"/>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="40"/>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="40"/>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="40"/>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="40"/>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="40"/>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="40"/>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="40"/>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="40"/>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="40"/>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="40"/>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="40"/>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="40"/>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="40"/>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="40"/>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
       <c r="D31" s="40"/>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
       <c r="D32" s="40"/>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>

</xml_diff>

<commit_message>
Update Project Plan for Checkpoint
</commit_message>
<xml_diff>
--- a/docs/project_plan.xlsx
+++ b/docs/project_plan.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\keanu\Desktop\CS2430\project3\Programming_Project_3\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BEED74C9-23CD-4E9E-8A99-620F78CF7A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EDE65C2-A42D-4DBA-801A-7A03A656F9C2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="24196" windowHeight="14476" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Info" sheetId="1" r:id="rId1"/>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="112">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="171" uniqueCount="131">
   <si>
     <t>CSIS 2430 — Project Plan (Plan + Trace)</t>
   </si>
@@ -77,9 +77,6 @@
   </si>
   <si>
     <t>Keanu Cruz</t>
-  </si>
-  <si>
-    <t>Communications Lead</t>
   </si>
   <si>
     <t>Assembles report/video; ensures run instructions; tracks deliverables; merges documentation.</t>
@@ -375,10 +372,71 @@
     <t>Greedy Fails Vs Brute Force</t>
   </si>
   <si>
-    <t>Matches Brute Force Optimal</t>
-  </si>
-  <si>
-    <t>Handles Large Dataset</t>
+    <t>Order Independence</t>
+  </si>
+  <si>
+    <t>Solver Immutable</t>
+  </si>
+  <si>
+    <t>Communications Lead (Inactive)</t>
+  </si>
+  <si>
+    <t>D</t>
+  </si>
+  <si>
+    <t>IP</t>
+  </si>
+  <si>
+    <t>e61faaf, PR#4</t>
+  </si>
+  <si>
+    <t>PR#4</t>
+  </si>
+  <si>
+    <t>PR#5</t>
+  </si>
+  <si>
+    <t>Submitted 4/5/2026</t>
+  </si>
+  <si>
+    <t>e61faaf</t>
+  </si>
+  <si>
+    <t>aa167c2, a8ff682</t>
+  </si>
+  <si>
+    <t>a8c3ab2</t>
+  </si>
+  <si>
+    <t>Issue#3</t>
+  </si>
+  <si>
+    <t>0c8127b, cb6381e</t>
+  </si>
+  <si>
+    <t>Done by Keanu</t>
+  </si>
+  <si>
+    <t>KnapsackSolver Deep Copy</t>
+  </si>
+  <si>
+    <t>Low</t>
+  </si>
+  <si>
+    <t>Issue#3 needs to be corrected</t>
+  </si>
+  <si>
+    <t>Code Implemented</t>
+  </si>
+  <si>
+    <t>Tests Implemented</t>
+  </si>
+  <si>
+    <t>Docs Present and Updated for Checkpoint</t>
+  </si>
+  <si>
+    <t xml:space="preserve">
+a47ba88</t>
   </si>
 </sst>
 </file>
@@ -388,13 +446,20 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="mm/dd/yy"/>
   </numFmts>
-  <fonts count="14" x14ac:knownFonts="1">
+  <fonts count="16" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -490,8 +555,14 @@
       <family val="2"/>
       <charset val="1"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="5">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -513,6 +584,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -632,118 +715,167 @@
   </borders>
   <cellStyleXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="9" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="10" fillId="2" borderId="0" applyBorder="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyBorder="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="54">
+  <cellXfs count="59">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="1" xfId="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="4" applyBorder="1" applyProtection="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="4" applyBorder="1" applyProtection="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="11" fillId="3" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="5" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="6" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -751,42 +883,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="2" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="4" borderId="0" xfId="3" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="5">
@@ -1068,14 +1164,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="18" x14ac:dyDescent="0.45">
-      <c r="A1" s="47" t="s">
+      <c r="A1" s="40" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="47"/>
-      <c r="C1" s="47"/>
-      <c r="D1" s="47"/>
-      <c r="E1" s="47"/>
-      <c r="F1" s="47"/>
+      <c r="B1" s="40"/>
+      <c r="C1" s="40"/>
+      <c r="D1" s="40"/>
+      <c r="E1" s="40"/>
+      <c r="F1" s="40"/>
     </row>
     <row r="3" spans="1:6" ht="15" x14ac:dyDescent="0.45">
       <c r="A3" s="2" t="s">
@@ -1094,81 +1190,81 @@
     </row>
     <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="B5" s="43"/>
-      <c r="C5" s="43"/>
-      <c r="D5" s="43"/>
-      <c r="E5" s="43"/>
-      <c r="F5" s="43"/>
+        <v>69</v>
+      </c>
+      <c r="B5" s="41"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="41"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="B6" s="43"/>
-      <c r="C6" s="43"/>
-      <c r="D6" s="43"/>
-      <c r="E6" s="43"/>
-      <c r="F6" s="43"/>
+        <v>70</v>
+      </c>
+      <c r="B6" s="41"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="41"/>
+      <c r="E6" s="41"/>
+      <c r="F6" s="41"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="B7" s="43"/>
-      <c r="C7" s="43"/>
-      <c r="D7" s="43"/>
-      <c r="E7" s="43"/>
-      <c r="F7" s="43"/>
+        <v>71</v>
+      </c>
+      <c r="B7" s="41"/>
+      <c r="C7" s="41"/>
+      <c r="D7" s="41"/>
+      <c r="E7" s="41"/>
+      <c r="F7" s="41"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="B8" s="43"/>
-      <c r="C8" s="43"/>
-      <c r="D8" s="43"/>
-      <c r="E8" s="43"/>
-      <c r="F8" s="43"/>
+        <v>72</v>
+      </c>
+      <c r="B8" s="41"/>
+      <c r="C8" s="41"/>
+      <c r="D8" s="41"/>
+      <c r="E8" s="41"/>
+      <c r="F8" s="41"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B9" s="43"/>
-      <c r="C9" s="43"/>
-      <c r="D9" s="43"/>
-      <c r="E9" s="43"/>
-      <c r="F9" s="43"/>
+        <v>73</v>
+      </c>
+      <c r="B9" s="41"/>
+      <c r="C9" s="41"/>
+      <c r="D9" s="41"/>
+      <c r="E9" s="41"/>
+      <c r="F9" s="41"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="4"/>
-      <c r="B10" s="43"/>
-      <c r="C10" s="43"/>
-      <c r="D10" s="43"/>
-      <c r="E10" s="43"/>
-      <c r="F10" s="43"/>
+      <c r="B10" s="41"/>
+      <c r="C10" s="41"/>
+      <c r="D10" s="41"/>
+      <c r="E10" s="41"/>
+      <c r="F10" s="41"/>
     </row>
     <row r="11" spans="1:6" ht="15" x14ac:dyDescent="0.45">
-      <c r="A11" s="46" t="s">
+      <c r="A11" s="42" t="s">
         <v>3</v>
       </c>
-      <c r="B11" s="46"/>
-      <c r="C11" s="46"/>
-      <c r="D11" s="46"/>
-      <c r="E11" s="46"/>
-      <c r="F11" s="46"/>
+      <c r="B11" s="42"/>
+      <c r="C11" s="42"/>
+      <c r="D11" s="42"/>
+      <c r="E11" s="42"/>
+      <c r="F11" s="42"/>
     </row>
     <row r="12" spans="1:6" ht="17.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A12" s="43" t="s">
+      <c r="A12" s="41" t="s">
         <v>4</v>
       </c>
-      <c r="B12" s="43"/>
-      <c r="C12" s="43"/>
-      <c r="D12" s="43"/>
-      <c r="E12" s="43"/>
-      <c r="F12" s="43"/>
+      <c r="B12" s="41"/>
+      <c r="C12" s="41"/>
+      <c r="D12" s="41"/>
+      <c r="E12" s="41"/>
+      <c r="F12" s="41"/>
     </row>
     <row r="13" spans="1:6" ht="18.75" customHeight="1" x14ac:dyDescent="0.45"/>
     <row r="14" spans="1:6" ht="30.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1187,25 +1283,25 @@
     </row>
     <row r="15" spans="1:6" ht="44.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="5" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="B15" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C15" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="D15" s="5"/>
     </row>
     <row r="16" spans="1:6" ht="45.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="5" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B16" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C16" s="5" t="s">
         <v>12</v>
-      </c>
-      <c r="C16" s="5" t="s">
-        <v>13</v>
       </c>
       <c r="D16" s="5"/>
     </row>
@@ -1220,118 +1316,103 @@
         <v>10</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="18" spans="1:4" ht="56.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="5" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B18" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C18" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="C18" s="5" t="s">
+      <c r="D18" s="5"/>
+    </row>
+    <row r="19" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="43" t="s">
         <v>16</v>
       </c>
-      <c r="D18" s="5"/>
-    </row>
-    <row r="19" spans="1:4" ht="31.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="44" t="s">
+      <c r="B19" s="43"/>
+    </row>
+    <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A20" s="41" t="s">
         <v>17</v>
       </c>
-      <c r="B19" s="44"/>
-    </row>
-    <row r="20" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A20" s="43" t="s">
+      <c r="B20" s="41"/>
+    </row>
+    <row r="21" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="41" t="s">
+        <v>77</v>
+      </c>
+      <c r="B21" s="41"/>
+    </row>
+    <row r="22" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A22" s="41" t="s">
+        <v>85</v>
+      </c>
+      <c r="B22" s="41"/>
+    </row>
+    <row r="23" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="B20" s="43"/>
-    </row>
-    <row r="21" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A21" s="43" t="s">
-        <v>78</v>
-      </c>
-      <c r="B21" s="43"/>
-    </row>
-    <row r="22" spans="1:4" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A22" s="50" t="s">
-        <v>86</v>
-      </c>
-      <c r="B22" s="50"/>
-    </row>
-    <row r="23" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="43" t="s">
+      <c r="B23" s="41"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A24" s="41"/>
+      <c r="B24" s="41"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
+      <c r="A25" s="43" t="s">
         <v>19</v>
       </c>
-      <c r="B23" s="43"/>
-    </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A24" s="43"/>
-      <c r="B24" s="43"/>
-    </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A25" s="44" t="s">
-        <v>20</v>
-      </c>
-      <c r="B25" s="44"/>
+      <c r="B25" s="43"/>
     </row>
     <row r="26" spans="1:4" ht="41.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A26" s="45" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B26" s="45"/>
     </row>
     <row r="27" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A27" s="44" t="s">
-        <v>21</v>
-      </c>
-      <c r="B27" s="44"/>
+      <c r="A27" s="43" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" s="43"/>
     </row>
     <row r="28" spans="1:4" ht="78.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" s="45" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" s="45"/>
+    </row>
+    <row r="29" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A29" s="44" t="s">
+        <v>78</v>
+      </c>
+      <c r="B29" s="44"/>
+    </row>
+    <row r="30" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A30" s="44" t="s">
+        <v>79</v>
+      </c>
+      <c r="B30" s="44"/>
+    </row>
+    <row r="31" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="A31" s="44" t="s">
         <v>22</v>
       </c>
-      <c r="B28" s="45"/>
-    </row>
-    <row r="29" spans="1:4" ht="18.75" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A29" s="42" t="s">
-        <v>79</v>
-      </c>
-      <c r="B29" s="42"/>
-    </row>
-    <row r="30" spans="1:4" ht="22.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A30" s="42" t="s">
-        <v>80</v>
-      </c>
-      <c r="B30" s="42"/>
-    </row>
-    <row r="31" spans="1:4" ht="20.25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A31" s="42" t="s">
-        <v>23</v>
-      </c>
-      <c r="B31" s="42"/>
+      <c r="B31" s="44"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
-      <c r="A32" s="43"/>
-      <c r="B32" s="43"/>
+      <c r="A32" s="41"/>
+      <c r="B32" s="41"/>
     </row>
   </sheetData>
   <mergeCells count="23">
-    <mergeCell ref="A1:F1"/>
-    <mergeCell ref="B5:F5"/>
-    <mergeCell ref="B6:F6"/>
-    <mergeCell ref="B7:F7"/>
-    <mergeCell ref="B8:F8"/>
-    <mergeCell ref="B9:F9"/>
-    <mergeCell ref="B10:F10"/>
-    <mergeCell ref="A11:F11"/>
-    <mergeCell ref="A12:F12"/>
-    <mergeCell ref="A19:B19"/>
-    <mergeCell ref="A20:B20"/>
-    <mergeCell ref="A21:B21"/>
-    <mergeCell ref="A22:B22"/>
-    <mergeCell ref="A23:B23"/>
-    <mergeCell ref="A24:B24"/>
     <mergeCell ref="A30:B30"/>
     <mergeCell ref="A31:B31"/>
     <mergeCell ref="A32:B32"/>
@@ -1340,6 +1421,21 @@
     <mergeCell ref="A27:B27"/>
     <mergeCell ref="A28:B28"/>
     <mergeCell ref="A29:B29"/>
+    <mergeCell ref="A20:B20"/>
+    <mergeCell ref="A21:B21"/>
+    <mergeCell ref="A22:B22"/>
+    <mergeCell ref="A23:B23"/>
+    <mergeCell ref="A24:B24"/>
+    <mergeCell ref="B9:F9"/>
+    <mergeCell ref="B10:F10"/>
+    <mergeCell ref="A11:F11"/>
+    <mergeCell ref="A12:F12"/>
+    <mergeCell ref="A19:B19"/>
+    <mergeCell ref="A1:F1"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B8:F8"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
@@ -1360,121 +1456,133 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="46" t="s">
+        <v>23</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+    </row>
+    <row r="2" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="47" t="s">
         <v>24</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-    </row>
-    <row r="2" spans="1:6" ht="19.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="49" t="s">
-        <v>25</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
     </row>
     <row r="4" spans="1:6" ht="27" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="B4" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="C4" s="8" t="s">
         <v>27</v>
       </c>
-      <c r="C4" s="8" t="s">
+      <c r="D4" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="D4" s="8" t="s">
+      <c r="E4" s="8" t="s">
         <v>29</v>
       </c>
-      <c r="E4" s="8" t="s">
+      <c r="F4" s="8" t="s">
         <v>30</v>
-      </c>
-      <c r="F4" s="8" t="s">
-        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:6" ht="27.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="10" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B5" s="11">
         <v>46110</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D5" s="10" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="12"/>
-      <c r="F5" s="10"/>
+        <v>32</v>
+      </c>
+      <c r="E5" s="12" t="s">
+        <v>112</v>
+      </c>
+      <c r="F5" s="10" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="6" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A6" s="10" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B6" s="11">
         <v>46117</v>
       </c>
       <c r="C6" s="10" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D6" s="10" t="s">
-        <v>35</v>
-      </c>
-      <c r="E6" s="12"/>
-      <c r="F6" s="10"/>
+        <v>34</v>
+      </c>
+      <c r="E6" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="7" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A7" s="10" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B7" s="11">
         <v>46117</v>
       </c>
       <c r="C7" s="10" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D7" s="10" t="s">
-        <v>37</v>
-      </c>
-      <c r="E7" s="12"/>
-      <c r="F7" s="10"/>
+        <v>36</v>
+      </c>
+      <c r="E7" s="12" t="s">
+        <v>113</v>
+      </c>
+      <c r="F7" s="10" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="8" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A8" s="10" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B8" s="11">
         <v>46123</v>
       </c>
       <c r="C8" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D8" s="10" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="E8" s="12"/>
       <c r="F8" s="10"/>
     </row>
     <row r="9" spans="1:6" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A9" s="10" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" s="11">
         <v>46124</v>
       </c>
       <c r="C9" s="10" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D9" s="10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E9" s="12"/>
       <c r="F9" s="10"/>
@@ -1503,53 +1611,53 @@
     <col min="1" max="1" width="6.06640625" customWidth="1"/>
     <col min="2" max="2" width="45.86328125" style="7" customWidth="1"/>
     <col min="3" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="29.46484375" style="36" customWidth="1"/>
+    <col min="6" max="6" width="29.46484375" style="35" customWidth="1"/>
     <col min="7" max="7" width="30" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="48" t="s">
+      <c r="A1" s="46" t="s">
+        <v>42</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+    </row>
+    <row r="2" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="47" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
-      <c r="F1" s="48"/>
-      <c r="G1" s="48"/>
-    </row>
-    <row r="2" spans="1:7" ht="16.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="49" t="s">
-        <v>44</v>
-      </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-      <c r="G2" s="49"/>
+      <c r="B2" s="47"/>
+      <c r="C2" s="47"/>
+      <c r="D2" s="47"/>
+      <c r="E2" s="47"/>
+      <c r="F2" s="47"/>
+      <c r="G2" s="47"/>
     </row>
     <row r="4" spans="1:7" ht="27" x14ac:dyDescent="0.45">
       <c r="A4" s="8" t="s">
+        <v>44</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="C4" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="D4" s="13" t="s">
         <v>46</v>
       </c>
-      <c r="C4" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="D4" s="13" t="s">
+      <c r="E4" s="13" t="s">
+        <v>29</v>
+      </c>
+      <c r="F4" s="30" t="s">
+        <v>30</v>
+      </c>
+      <c r="G4" s="13" t="s">
         <v>47</v>
-      </c>
-      <c r="E4" s="13" t="s">
-        <v>30</v>
-      </c>
-      <c r="F4" s="30" t="s">
-        <v>31</v>
-      </c>
-      <c r="G4" s="13" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="5" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1557,16 +1665,20 @@
         <v>1</v>
       </c>
       <c r="B5" s="15" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C5" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D5" s="16">
         <v>46110</v>
       </c>
-      <c r="E5" s="17"/>
-      <c r="F5" s="31"/>
+      <c r="E5" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F5" s="49" t="s">
+        <v>119</v>
+      </c>
       <c r="G5" s="15"/>
     </row>
     <row r="6" spans="1:7" ht="31.15" customHeight="1" x14ac:dyDescent="0.45">
@@ -1574,16 +1686,20 @@
         <v>2</v>
       </c>
       <c r="B6" s="15" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C6" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D6" s="16">
         <v>46117</v>
       </c>
-      <c r="E6" s="17"/>
-      <c r="F6" s="32"/>
+      <c r="E6" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F6" s="31" t="s">
+        <v>115</v>
+      </c>
       <c r="G6" s="15"/>
     </row>
     <row r="7" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1591,16 +1707,18 @@
         <v>3</v>
       </c>
       <c r="B7" s="15" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C7" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D7" s="16">
         <v>46123</v>
       </c>
-      <c r="E7" s="17"/>
-      <c r="F7" s="32"/>
+      <c r="E7" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="F7" s="31"/>
       <c r="G7" s="15"/>
     </row>
     <row r="8" spans="1:7" ht="33.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1608,16 +1726,16 @@
         <v>4</v>
       </c>
       <c r="B8" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C8" s="15" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D8" s="16">
         <v>46123</v>
       </c>
       <c r="E8" s="17"/>
-      <c r="F8" s="33"/>
+      <c r="F8" s="32"/>
       <c r="G8" s="15"/>
     </row>
     <row r="9" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1625,16 +1743,20 @@
         <v>5</v>
       </c>
       <c r="B9" s="15" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C9" s="15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D9" s="16">
         <v>46110</v>
       </c>
-      <c r="E9" s="17"/>
-      <c r="F9" s="34"/>
+      <c r="E9" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F9" s="48" t="s">
+        <v>120</v>
+      </c>
       <c r="G9" s="15"/>
     </row>
     <row r="10" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1642,16 +1764,20 @@
         <v>6</v>
       </c>
       <c r="B10" s="15" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C10" s="15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D10" s="16">
         <v>46117</v>
       </c>
-      <c r="E10" s="17"/>
-      <c r="F10" s="34"/>
+      <c r="E10" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F10" s="48" t="s">
+        <v>116</v>
+      </c>
       <c r="G10" s="15"/>
     </row>
     <row r="11" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1659,16 +1785,20 @@
         <v>7</v>
       </c>
       <c r="B11" s="15" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C11" s="15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D11" s="16">
         <v>46123</v>
       </c>
-      <c r="E11" s="17"/>
-      <c r="F11" s="34"/>
+      <c r="E11" s="17" t="s">
+        <v>113</v>
+      </c>
+      <c r="F11" s="48" t="s">
+        <v>121</v>
+      </c>
       <c r="G11" s="15"/>
     </row>
     <row r="12" spans="1:7" ht="26.85" customHeight="1" x14ac:dyDescent="0.45">
@@ -1676,16 +1806,16 @@
         <v>8</v>
       </c>
       <c r="B12" s="18" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C12" s="15" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D12" s="16">
         <v>46123</v>
       </c>
       <c r="E12" s="17"/>
-      <c r="F12" s="34"/>
+      <c r="F12" s="33"/>
       <c r="G12" s="15"/>
     </row>
     <row r="13" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1693,67 +1823,85 @@
         <v>9</v>
       </c>
       <c r="B13" s="15" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C13" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D13" s="16">
         <v>46110</v>
       </c>
-      <c r="E13" s="17"/>
-      <c r="F13" s="34"/>
-      <c r="G13" s="15"/>
+      <c r="E13" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F13" s="48" t="s">
+        <v>122</v>
+      </c>
+      <c r="G13" s="15" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="14" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="14">
         <v>10</v>
       </c>
       <c r="B14" s="15" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C14" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D14" s="16">
         <v>46117</v>
       </c>
-      <c r="E14" s="17"/>
-      <c r="F14" s="34"/>
-      <c r="G14" s="15"/>
+      <c r="E14" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F14" s="50" t="s">
+        <v>118</v>
+      </c>
+      <c r="G14" s="15" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="15" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="14">
         <v>11</v>
       </c>
       <c r="B15" s="15" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C15" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D15" s="16">
         <v>46117</v>
       </c>
-      <c r="E15" s="17"/>
-      <c r="F15" s="34"/>
-      <c r="G15" s="15"/>
+      <c r="E15" s="17" t="s">
+        <v>112</v>
+      </c>
+      <c r="F15" s="48" t="s">
+        <v>117</v>
+      </c>
+      <c r="G15" s="15" t="s">
+        <v>123</v>
+      </c>
     </row>
     <row r="16" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="19">
         <v>12</v>
       </c>
       <c r="B16" s="18" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C16" s="15" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D16" s="16">
         <v>46124</v>
       </c>
       <c r="E16" s="17"/>
-      <c r="F16" s="34"/>
+      <c r="F16" s="33"/>
       <c r="G16" s="15"/>
     </row>
     <row r="17" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1762,7 +1910,7 @@
       <c r="C17" s="21"/>
       <c r="D17" s="22"/>
       <c r="E17" s="23"/>
-      <c r="F17" s="35"/>
+      <c r="F17" s="34"/>
       <c r="G17" s="22"/>
     </row>
     <row r="18" spans="1:7" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
@@ -1771,7 +1919,7 @@
       <c r="C18" s="15"/>
       <c r="D18" s="15"/>
       <c r="E18" s="17"/>
-      <c r="F18" s="34"/>
+      <c r="F18" s="33"/>
       <c r="G18" s="15"/>
     </row>
   </sheetData>
@@ -1780,7 +1928,7 @@
     <mergeCell ref="A2:G2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1796,177 +1944,177 @@
   <sheetData>
     <row r="1" spans="1:2" ht="19.5" x14ac:dyDescent="0.6">
       <c r="A1" s="24" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="2" spans="1:2" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" s="41" t="s">
+      <c r="A2" s="51" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A3" s="51" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A4" s="51" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A5" s="51" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A6" s="51" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A7" s="51" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A8" s="51" t="s">
         <v>91</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A3" s="41" t="s">
-        <v>87</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A4" s="41" t="s">
-        <v>88</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A5" s="41" t="s">
-        <v>107</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A6" s="41" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A7" s="41" t="s">
-        <v>90</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A8" s="41" t="s">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A9" s="51" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A9" s="41" t="s">
-        <v>93</v>
-      </c>
-    </row>
     <row r="10" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A10" s="41" t="s">
+      <c r="A10" s="51" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A11" s="51" t="s">
         <v>102</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A11" s="41" t="s">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A12" s="52" t="s">
         <v>103</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A12" s="53" t="s">
-        <v>104</v>
       </c>
     </row>
     <row r="13" spans="1:2" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A13" s="24" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="14" spans="1:2" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A14" s="51" t="s">
-        <v>91</v>
+      <c r="A14" s="53" t="s">
+        <v>90</v>
       </c>
     </row>
     <row r="15" spans="1:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A15" s="52" t="s">
+      <c r="A15" s="54" t="s">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
+      <c r="A16" s="53" t="s">
+        <v>96</v>
+      </c>
+      <c r="B16" s="25"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A17" s="53" t="s">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A18" s="53" t="s">
         <v>99</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.45">
-      <c r="A16" s="51" t="s">
-        <v>97</v>
-      </c>
-      <c r="B16" s="25"/>
-    </row>
-    <row r="17" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A17" s="51" t="s">
-        <v>98</v>
-      </c>
-    </row>
-    <row r="18" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A18" s="51" t="s">
+    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A19" s="53" t="s">
         <v>100</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A19" s="51" t="s">
-        <v>101</v>
-      </c>
-    </row>
     <row r="20" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A20" s="51" t="s">
-        <v>108</v>
+      <c r="A20" s="53" t="s">
+        <v>107</v>
       </c>
     </row>
     <row r="21" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A21" s="52"/>
+      <c r="A21" s="54" t="s">
+        <v>109</v>
+      </c>
     </row>
     <row r="22" spans="1:1" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A22" s="24" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="23" spans="1:1" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
+      <c r="A23" s="53" t="s">
         <v>95</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="23.25" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A23" s="51" t="s">
-        <v>96</v>
-      </c>
-    </row>
     <row r="24" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A24" s="51" t="s">
+      <c r="A24" s="53" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
+      <c r="A25" s="53" t="s">
         <v>105</v>
       </c>
     </row>
-    <row r="25" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A25" s="51" t="s">
-        <v>106</v>
-      </c>
-    </row>
     <row r="26" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A26" s="51" t="s">
-        <v>109</v>
+      <c r="A26" s="53" t="s">
+        <v>108</v>
       </c>
     </row>
     <row r="27" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A27" s="51"/>
+      <c r="A27" s="39" t="s">
+        <v>110</v>
+      </c>
     </row>
     <row r="28" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A28" s="51"/>
+      <c r="A28" s="55"/>
     </row>
     <row r="29" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A29" s="51"/>
+      <c r="A29" s="55"/>
     </row>
     <row r="30" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A30" s="52"/>
+      <c r="A30" s="56"/>
     </row>
     <row r="31" spans="1:1" ht="19.899999999999999" thickBot="1" x14ac:dyDescent="0.65">
       <c r="A31" s="24" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="32" spans="1:1" ht="21.75" customHeight="1" thickTop="1" x14ac:dyDescent="0.45">
-      <c r="A32" s="51" t="s">
-        <v>110</v>
-      </c>
+      <c r="A32" s="55"/>
     </row>
     <row r="33" spans="1:1" ht="15.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A33" s="51" t="s">
-        <v>111</v>
-      </c>
+      <c r="A33" s="55"/>
     </row>
     <row r="34" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A34" s="51"/>
+      <c r="A34" s="55"/>
     </row>
     <row r="35" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A35" s="51"/>
+      <c r="A35" s="55"/>
     </row>
     <row r="36" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A36" s="51"/>
+      <c r="A36" s="55"/>
     </row>
     <row r="37" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A37" s="51"/>
+      <c r="A37" s="55"/>
     </row>
     <row r="38" spans="1:1" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A38" s="51"/>
+      <c r="A38" s="55"/>
     </row>
     <row r="39" spans="1:1" x14ac:dyDescent="0.45">
-      <c r="A39" s="52"/>
+      <c r="A39" s="56"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -1987,37 +2135,47 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="48" t="s">
-        <v>60</v>
-      </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
-      <c r="E1" s="48"/>
+      <c r="A1" s="46" t="s">
+        <v>59</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A3" s="8" t="s">
+        <v>60</v>
+      </c>
+      <c r="B3" s="8" t="s">
         <v>61</v>
       </c>
-      <c r="B3" s="8" t="s">
+      <c r="C3" s="8" t="s">
         <v>62</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="8" t="s">
+        <v>27</v>
+      </c>
+      <c r="E3" s="8" t="s">
         <v>63</v>
       </c>
-      <c r="D3" s="8" t="s">
-        <v>28</v>
-      </c>
-      <c r="E3" s="8" t="s">
-        <v>64</v>
-      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.45">
-      <c r="A4" s="26"/>
-      <c r="B4" s="26"/>
-      <c r="C4" s="26"/>
-      <c r="D4" s="26"/>
-      <c r="E4" s="26"/>
+      <c r="A4" s="26" t="s">
+        <v>124</v>
+      </c>
+      <c r="B4" s="26" t="s">
+        <v>125</v>
+      </c>
+      <c r="C4" s="26" t="s">
+        <v>126</v>
+      </c>
+      <c r="D4" s="26" t="s">
+        <v>80</v>
+      </c>
+      <c r="E4" s="26" t="s">
+        <v>113</v>
+      </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="26"/>
@@ -2050,210 +2208,228 @@
     <col min="1" max="1" width="14" customWidth="1"/>
     <col min="2" max="2" width="52.06640625" customWidth="1"/>
     <col min="3" max="3" width="34" customWidth="1"/>
-    <col min="4" max="4" width="28.9296875" style="36" customWidth="1"/>
+    <col min="4" max="4" width="28.9296875" style="35" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" ht="15.4" x14ac:dyDescent="0.45">
-      <c r="A1" s="48" t="s">
-        <v>65</v>
-      </c>
-      <c r="B1" s="48"/>
-      <c r="C1" s="48"/>
-      <c r="D1" s="48"/>
+      <c r="A1" s="46" t="s">
+        <v>64</v>
+      </c>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A3" s="27" t="s">
+        <v>65</v>
+      </c>
+      <c r="B3" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="B3" s="27" t="s">
+      <c r="C3" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="C3" s="27" t="s">
+      <c r="D3" s="36" t="s">
         <v>68</v>
       </c>
-      <c r="D3" s="37" t="s">
-        <v>69</v>
-      </c>
     </row>
     <row r="4" spans="1:4" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A4" s="28"/>
-      <c r="B4" s="29"/>
+      <c r="A4" s="28">
+        <v>46116</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>127</v>
+      </c>
       <c r="C4" s="29"/>
-      <c r="D4" s="38"/>
+      <c r="D4" s="57" t="s">
+        <v>115</v>
+      </c>
     </row>
     <row r="5" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A5" s="28"/>
-      <c r="B5" s="29"/>
+      <c r="A5" s="28">
+        <v>46116</v>
+      </c>
+      <c r="B5" s="29" t="s">
+        <v>128</v>
+      </c>
       <c r="C5" s="29"/>
-      <c r="D5" s="38"/>
+      <c r="D5" s="57" t="s">
+        <v>116</v>
+      </c>
     </row>
     <row r="6" spans="1:4" ht="34.5" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A6" s="28"/>
-      <c r="B6" s="29"/>
+      <c r="A6" s="28">
+        <v>46117</v>
+      </c>
+      <c r="B6" s="29" t="s">
+        <v>129</v>
+      </c>
       <c r="C6" s="29"/>
-      <c r="D6" s="39"/>
+      <c r="D6" s="58" t="s">
+        <v>130</v>
+      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A7" s="28"/>
       <c r="B7" s="10"/>
       <c r="C7" s="10"/>
-      <c r="D7" s="39"/>
+      <c r="D7" s="37"/>
     </row>
     <row r="8" spans="1:4" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="10"/>
       <c r="B8" s="10"/>
       <c r="C8" s="10"/>
-      <c r="D8" s="39"/>
+      <c r="D8" s="37"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A9" s="10"/>
       <c r="B9" s="10"/>
       <c r="C9" s="10"/>
-      <c r="D9" s="39"/>
+      <c r="D9" s="37"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A10" s="1"/>
       <c r="B10" s="1"/>
       <c r="C10" s="1"/>
-      <c r="D10" s="40"/>
+      <c r="D10" s="38"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A11" s="1"/>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
-      <c r="D11" s="40"/>
+      <c r="D11" s="38"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A12" s="1"/>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
-      <c r="D12" s="40"/>
+      <c r="D12" s="38"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A13" s="1"/>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
-      <c r="D13" s="40"/>
+      <c r="D13" s="38"/>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A14" s="1"/>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
-      <c r="D14" s="40"/>
+      <c r="D14" s="38"/>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A15" s="1"/>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
-      <c r="D15" s="40"/>
+      <c r="D15" s="38"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A16" s="1"/>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
-      <c r="D16" s="40"/>
+      <c r="D16" s="38"/>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A17" s="1"/>
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
-      <c r="D17" s="40"/>
+      <c r="D17" s="38"/>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A18" s="1"/>
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
-      <c r="D18" s="40"/>
+      <c r="D18" s="38"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A19" s="1"/>
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
-      <c r="D19" s="40"/>
+      <c r="D19" s="38"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A20" s="1"/>
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
-      <c r="D20" s="40"/>
+      <c r="D20" s="38"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A21" s="1"/>
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
-      <c r="D21" s="40"/>
+      <c r="D21" s="38"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A22" s="1"/>
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
-      <c r="D22" s="40"/>
+      <c r="D22" s="38"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A23" s="1"/>
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
-      <c r="D23" s="40"/>
+      <c r="D23" s="38"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A24" s="1"/>
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
-      <c r="D24" s="40"/>
+      <c r="D24" s="38"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A25" s="1"/>
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
-      <c r="D25" s="40"/>
+      <c r="D25" s="38"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A26" s="1"/>
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
-      <c r="D26" s="40"/>
+      <c r="D26" s="38"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A27" s="1"/>
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
-      <c r="D27" s="40"/>
+      <c r="D27" s="38"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A28" s="1"/>
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
-      <c r="D28" s="40"/>
+      <c r="D28" s="38"/>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A29" s="1"/>
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
-      <c r="D29" s="40"/>
+      <c r="D29" s="38"/>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A30" s="1"/>
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
-      <c r="D30" s="40"/>
+      <c r="D30" s="38"/>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A31" s="1"/>
       <c r="B31" s="1"/>
       <c r="C31" s="1"/>
-      <c r="D31" s="40"/>
+      <c r="D31" s="38"/>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A32" s="1"/>
       <c r="B32" s="1"/>
       <c r="C32" s="1"/>
-      <c r="D32" s="40"/>
+      <c r="D32" s="38"/>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.45">
       <c r="A33" s="1"/>
       <c r="B33" s="1"/>
       <c r="C33" s="1"/>
-      <c r="D33" s="40"/>
+      <c r="D33" s="38"/>
     </row>
   </sheetData>
   <mergeCells count="1">

</xml_diff>